<commit_message>
Update Excel template to remove stock take sheet
Remove the "Weekly Stock Take" sheet from the Excel export and update the metadata title.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: a3bb658e-c1b8-4d25-a4e2-55594f80be40
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: db6813cb-301f-4002-abc9-54c9821f830f
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9fb187d0-5a71-40d4-a291-96ab5e107c04/a3bb658e-c1b8-4d25-a4e2-55594f80be40/IeCay9D
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/silo-tracker/public/silo-mate-feed-program.xlsx
+++ b/artifacts/silo-tracker/public/silo-mate-feed-program.xlsx
@@ -11,15 +11,14 @@
     <sheet sheetId="5" name="SHED 7 &amp; 8" state="visible" r:id="rId8"/>
     <sheet sheetId="6" name="SHED 9 &amp; 10" state="visible" r:id="rId9"/>
     <sheet sheetId="7" name="SHED 11 &amp; 12" state="visible" r:id="rId10"/>
-    <sheet sheetId="8" name="WEEKLY STOCK TAKE" state="visible" r:id="rId11"/>
-    <sheet sheetId="9" name="end of batch" state="visible" r:id="rId12"/>
+    <sheet sheetId="8" name="end of batch" state="visible" r:id="rId11"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="591" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="538" uniqueCount="105">
   <si>
     <t xml:space="preserve">    AGE</t>
   </si>
@@ -244,45 +243,6 @@
   </si>
   <si>
     <t>shed 12</t>
-  </si>
-  <si>
-    <t>FEED STOCKTAKE</t>
-  </si>
-  <si>
-    <t>Date:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FARM:  </t>
-  </si>
-  <si>
-    <t>double b</t>
-  </si>
-  <si>
-    <t>Monday</t>
-  </si>
-  <si>
-    <t>Tuesday</t>
-  </si>
-  <si>
-    <t>Wednesday</t>
-  </si>
-  <si>
-    <t>Thursday</t>
-  </si>
-  <si>
-    <t>Friday</t>
-  </si>
-  <si>
-    <t>SHEDS</t>
-  </si>
-  <si>
-    <t>FEED TYPE</t>
-  </si>
-  <si>
-    <t>FEED IN STOCK (kg)</t>
-  </si>
-  <si>
-    <t>starter</t>
   </si>
   <si>
     <t xml:space="preserve">Farm </t>
@@ -861,7 +821,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="119">
+  <cellXfs count="113">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1075,39 +1035,6 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="6" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="6" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1116,6 +1043,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="4" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1126,7 +1056,13 @@
     <xf numFmtId="2" fontId="4" fillId="8" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="167" fontId="4" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1143,6 +1079,12 @@
     </xf>
     <xf numFmtId="2" fontId="4" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -29967,500 +29909,6 @@
   <sheetPr>
     <tabColor rgb="FF217346"/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="6" customWidth="1"/>
-    <col min="2" max="2" width="17" customWidth="1"/>
-    <col min="3" max="3" width="13" customWidth="1"/>
-    <col min="4" max="4" width="21" customWidth="1"/>
-    <col min="5" max="9" width="17" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="40" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="90"/>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-      <c r="I1" s="90"/>
-    </row>
-    <row r="2" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="7"/>
-      <c r="B2" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F2" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="3" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="29"/>
-      <c r="B3" s="30" t="s">
-        <v>76</v>
-      </c>
-      <c r="C3" s="91"/>
-      <c r="D3" s="91"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="30"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="30"/>
-      <c r="I3" s="34"/>
-    </row>
-    <row r="4" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="29"/>
-      <c r="B4" s="30" t="s">
-        <v>77</v>
-      </c>
-      <c r="C4" s="92" t="s">
-        <v>78</v>
-      </c>
-      <c r="D4" s="30" t="s">
-        <v>78</v>
-      </c>
-      <c r="E4" s="30" t="s">
-        <v>79</v>
-      </c>
-      <c r="F4" s="30" t="s">
-        <v>80</v>
-      </c>
-      <c r="G4" s="30" t="s">
-        <v>81</v>
-      </c>
-      <c r="H4" s="30" t="s">
-        <v>82</v>
-      </c>
-      <c r="I4" s="34" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="5" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="29"/>
-      <c r="B5" s="30" t="s">
-        <v>84</v>
-      </c>
-      <c r="C5" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="D5" s="30" t="s">
-        <v>85</v>
-      </c>
-      <c r="E5" s="30" t="s">
-        <v>86</v>
-      </c>
-      <c r="F5" s="30" t="s">
-        <v>86</v>
-      </c>
-      <c r="G5" s="30" t="s">
-        <v>86</v>
-      </c>
-      <c r="H5" s="30" t="s">
-        <v>86</v>
-      </c>
-      <c r="I5" s="34" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="93"/>
-      <c r="B6" s="94" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="95" t="s">
-        <v>47</v>
-      </c>
-      <c r="D6" s="95" t="s">
-        <v>87</v>
-      </c>
-      <c r="E6" s="95"/>
-      <c r="F6" s="95"/>
-      <c r="G6" s="71">
-        <v>18000</v>
-      </c>
-      <c r="H6" s="95"/>
-      <c r="I6" s="96"/>
-    </row>
-    <row r="7" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="97"/>
-      <c r="B7" s="62"/>
-      <c r="C7" s="62" t="s">
-        <v>48</v>
-      </c>
-      <c r="D7" s="62"/>
-      <c r="E7" s="62"/>
-      <c r="F7" s="62"/>
-      <c r="G7" s="61">
-        <v>24000</v>
-      </c>
-      <c r="H7" s="62"/>
-      <c r="I7" s="98"/>
-    </row>
-    <row r="8" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="93"/>
-      <c r="B8" s="95"/>
-      <c r="C8" s="95" t="s">
-        <v>49</v>
-      </c>
-      <c r="D8" s="95"/>
-      <c r="E8" s="95"/>
-      <c r="F8" s="95"/>
-      <c r="G8" s="71">
-        <v>8000</v>
-      </c>
-      <c r="H8" s="95"/>
-      <c r="I8" s="96"/>
-    </row>
-    <row r="9" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="97"/>
-      <c r="B9" s="62"/>
-      <c r="C9" s="62"/>
-      <c r="D9" s="62"/>
-      <c r="E9" s="62"/>
-      <c r="F9" s="62"/>
-      <c r="G9" s="62"/>
-      <c r="H9" s="62"/>
-      <c r="I9" s="98"/>
-    </row>
-    <row r="10" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="93"/>
-      <c r="B10" s="94" t="s">
-        <v>58</v>
-      </c>
-      <c r="C10" s="95" t="s">
-        <v>47</v>
-      </c>
-      <c r="D10" s="95"/>
-      <c r="E10" s="95"/>
-      <c r="F10" s="95"/>
-      <c r="G10" s="71">
-        <v>19000</v>
-      </c>
-      <c r="H10" s="95"/>
-      <c r="I10" s="96"/>
-    </row>
-    <row r="11" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="97"/>
-      <c r="B11" s="62"/>
-      <c r="C11" s="62" t="s">
-        <v>48</v>
-      </c>
-      <c r="D11" s="62"/>
-      <c r="E11" s="62"/>
-      <c r="F11" s="62"/>
-      <c r="G11" s="61">
-        <v>24000</v>
-      </c>
-      <c r="H11" s="62"/>
-      <c r="I11" s="98"/>
-    </row>
-    <row r="12" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="93"/>
-      <c r="B12" s="95"/>
-      <c r="C12" s="95" t="s">
-        <v>49</v>
-      </c>
-      <c r="D12" s="95"/>
-      <c r="E12" s="95"/>
-      <c r="F12" s="95"/>
-      <c r="G12" s="71">
-        <v>8000</v>
-      </c>
-      <c r="H12" s="95"/>
-      <c r="I12" s="96"/>
-    </row>
-    <row r="13" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="97"/>
-      <c r="B13" s="62"/>
-      <c r="C13" s="62"/>
-      <c r="D13" s="62"/>
-      <c r="E13" s="62"/>
-      <c r="F13" s="62"/>
-      <c r="G13" s="62"/>
-      <c r="H13" s="62"/>
-      <c r="I13" s="98"/>
-    </row>
-    <row r="14" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="93"/>
-      <c r="B14" s="94" t="s">
-        <v>61</v>
-      </c>
-      <c r="C14" s="95" t="s">
-        <v>47</v>
-      </c>
-      <c r="D14" s="95"/>
-      <c r="E14" s="95"/>
-      <c r="F14" s="95"/>
-      <c r="G14" s="71">
-        <v>8000</v>
-      </c>
-      <c r="H14" s="95"/>
-      <c r="I14" s="96"/>
-    </row>
-    <row r="15" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="97"/>
-      <c r="B15" s="62"/>
-      <c r="C15" s="62" t="s">
-        <v>48</v>
-      </c>
-      <c r="D15" s="62"/>
-      <c r="E15" s="62"/>
-      <c r="F15" s="62"/>
-      <c r="G15" s="61">
-        <v>22000</v>
-      </c>
-      <c r="H15" s="62"/>
-      <c r="I15" s="98"/>
-    </row>
-    <row r="16" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="93"/>
-      <c r="B16" s="95"/>
-      <c r="C16" s="95" t="s">
-        <v>49</v>
-      </c>
-      <c r="D16" s="95"/>
-      <c r="E16" s="95"/>
-      <c r="F16" s="95"/>
-      <c r="G16" s="71">
-        <v>24000</v>
-      </c>
-      <c r="H16" s="95"/>
-      <c r="I16" s="96"/>
-    </row>
-    <row r="17" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="97"/>
-      <c r="B17" s="62"/>
-      <c r="C17" s="62"/>
-      <c r="D17" s="62"/>
-      <c r="E17" s="62"/>
-      <c r="F17" s="62"/>
-      <c r="G17" s="62"/>
-      <c r="H17" s="62"/>
-      <c r="I17" s="98"/>
-    </row>
-    <row r="18" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="93"/>
-      <c r="B18" s="94" t="s">
-        <v>64</v>
-      </c>
-      <c r="C18" s="95" t="s">
-        <v>47</v>
-      </c>
-      <c r="D18" s="95"/>
-      <c r="E18" s="95"/>
-      <c r="F18" s="95"/>
-      <c r="G18" s="71">
-        <v>26000</v>
-      </c>
-      <c r="H18" s="95"/>
-      <c r="I18" s="96"/>
-    </row>
-    <row r="19" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="97"/>
-      <c r="B19" s="62"/>
-      <c r="C19" s="62" t="s">
-        <v>48</v>
-      </c>
-      <c r="D19" s="62"/>
-      <c r="E19" s="62"/>
-      <c r="F19" s="62"/>
-      <c r="G19" s="61">
-        <v>14000</v>
-      </c>
-      <c r="H19" s="62"/>
-      <c r="I19" s="98"/>
-    </row>
-    <row r="20" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="93"/>
-      <c r="B20" s="95"/>
-      <c r="C20" s="95" t="s">
-        <v>49</v>
-      </c>
-      <c r="D20" s="95"/>
-      <c r="E20" s="95"/>
-      <c r="F20" s="95"/>
-      <c r="G20" s="71">
-        <v>20000</v>
-      </c>
-      <c r="H20" s="95"/>
-      <c r="I20" s="96"/>
-    </row>
-    <row r="21" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="97"/>
-      <c r="B21" s="62"/>
-      <c r="C21" s="62"/>
-      <c r="D21" s="62"/>
-      <c r="E21" s="62"/>
-      <c r="F21" s="62"/>
-      <c r="G21" s="62"/>
-      <c r="H21" s="62"/>
-      <c r="I21" s="98"/>
-    </row>
-    <row r="22" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="93"/>
-      <c r="B22" s="94" t="s">
-        <v>67</v>
-      </c>
-      <c r="C22" s="95" t="s">
-        <v>47</v>
-      </c>
-      <c r="D22" s="95"/>
-      <c r="E22" s="95"/>
-      <c r="F22" s="95"/>
-      <c r="G22" s="71">
-        <v>26000</v>
-      </c>
-      <c r="H22" s="95"/>
-      <c r="I22" s="96"/>
-    </row>
-    <row r="23" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="97"/>
-      <c r="B23" s="62"/>
-      <c r="C23" s="62" t="s">
-        <v>48</v>
-      </c>
-      <c r="D23" s="62"/>
-      <c r="E23" s="62"/>
-      <c r="F23" s="62"/>
-      <c r="G23" s="61">
-        <v>14000</v>
-      </c>
-      <c r="H23" s="62"/>
-      <c r="I23" s="98"/>
-    </row>
-    <row r="24" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="93"/>
-      <c r="B24" s="95"/>
-      <c r="C24" s="95" t="s">
-        <v>49</v>
-      </c>
-      <c r="D24" s="95"/>
-      <c r="E24" s="95"/>
-      <c r="F24" s="95"/>
-      <c r="G24" s="95"/>
-      <c r="H24" s="95"/>
-      <c r="I24" s="96"/>
-    </row>
-    <row r="25" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="97"/>
-      <c r="B25" s="62"/>
-      <c r="C25" s="62"/>
-      <c r="D25" s="62"/>
-      <c r="E25" s="62"/>
-      <c r="F25" s="62"/>
-      <c r="G25" s="62"/>
-      <c r="H25" s="62"/>
-      <c r="I25" s="98"/>
-    </row>
-    <row r="26" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="93"/>
-      <c r="B26" s="94" t="s">
-        <v>70</v>
-      </c>
-      <c r="C26" s="95" t="s">
-        <v>47</v>
-      </c>
-      <c r="D26" s="95"/>
-      <c r="E26" s="95"/>
-      <c r="F26" s="95"/>
-      <c r="G26" s="71">
-        <v>26000</v>
-      </c>
-      <c r="H26" s="95"/>
-      <c r="I26" s="96"/>
-    </row>
-    <row r="27" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="97"/>
-      <c r="B27" s="62"/>
-      <c r="C27" s="62" t="s">
-        <v>48</v>
-      </c>
-      <c r="D27" s="62"/>
-      <c r="E27" s="62"/>
-      <c r="F27" s="62"/>
-      <c r="G27" s="61">
-        <v>14000</v>
-      </c>
-      <c r="H27" s="62"/>
-      <c r="I27" s="98"/>
-    </row>
-    <row r="28" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="93"/>
-      <c r="B28" s="95"/>
-      <c r="C28" s="95" t="s">
-        <v>49</v>
-      </c>
-      <c r="D28" s="95"/>
-      <c r="E28" s="95"/>
-      <c r="F28" s="95"/>
-      <c r="G28" s="71">
-        <v>14000</v>
-      </c>
-      <c r="H28" s="95"/>
-      <c r="I28" s="96"/>
-    </row>
-    <row r="29" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="97"/>
-      <c r="B29" s="62"/>
-      <c r="C29" s="62"/>
-      <c r="D29" s="62"/>
-      <c r="E29" s="62"/>
-      <c r="F29" s="62"/>
-      <c r="G29" s="62"/>
-      <c r="H29" s="62"/>
-      <c r="I29" s="98"/>
-    </row>
-    <row r="30" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="99"/>
-      <c r="B30" s="100" t="s">
-        <v>28</v>
-      </c>
-      <c r="C30" s="100" t="s">
-        <v>28</v>
-      </c>
-      <c r="D30" s="100" t="s">
-        <v>28</v>
-      </c>
-      <c r="E30" s="100"/>
-      <c r="F30" s="100"/>
-      <c r="G30" s="100"/>
-      <c r="H30" s="100"/>
-      <c r="I30" s="101">
-        <f>SUM(I7:I29)</f>
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <tabColor rgb="FF217346"/>
-  </sheetPr>
   <dimension ref="A1:Y37"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -30488,63 +29936,63 @@
   <sheetData>
     <row r="1" ht="40" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="90" t="s">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="B1" s="90" t="s">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="C1" s="90" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="D1" s="90"/>
       <c r="E1" s="90"/>
       <c r="F1" s="90" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="G1" s="90" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="H1" s="90" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="I1" s="90" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="J1" s="90" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="K1" s="90" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="L1" s="90" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="M1" s="90" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="N1" s="90" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="O1" s="90" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="P1" s="90" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="Q1" s="90" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="R1" s="90" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="S1" s="90" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="T1" s="90" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="U1" s="90" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="V1" s="90"/>
       <c r="W1" s="90"/>
@@ -30553,10 +30001,10 @@
     </row>
     <row r="2" ht="28" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="C2" s="7">
         <v>119</v>
@@ -30589,210 +30037,210 @@
       <c r="Y2" s="7"/>
     </row>
     <row r="3" ht="24" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A3" s="102"/>
+      <c r="A3" s="91"/>
       <c r="B3" s="30" t="s">
+        <v>78</v>
+      </c>
+      <c r="C3" s="30" t="s">
+        <v>78</v>
+      </c>
+      <c r="D3" s="92">
+        <v>114</v>
+      </c>
+      <c r="E3" s="92">
+        <v>114</v>
+      </c>
+      <c r="F3" s="92">
+        <v>114</v>
+      </c>
+      <c r="G3" s="92">
+        <v>114</v>
+      </c>
+      <c r="H3" s="92"/>
+      <c r="I3" s="92"/>
+      <c r="J3" s="92"/>
+      <c r="K3" s="92"/>
+      <c r="L3" s="92"/>
+      <c r="M3" s="92"/>
+      <c r="N3" s="92"/>
+      <c r="O3" s="92"/>
+      <c r="P3" s="92"/>
+      <c r="Q3" s="92"/>
+      <c r="R3" s="92"/>
+      <c r="S3" s="92"/>
+      <c r="T3" s="92"/>
+      <c r="U3" s="92"/>
+      <c r="V3" s="30" t="s">
+        <v>79</v>
+      </c>
+      <c r="W3" s="30" t="s">
+        <v>79</v>
+      </c>
+      <c r="X3" s="30" t="s">
+        <v>79</v>
+      </c>
+      <c r="Y3" s="30" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A4" s="91"/>
+      <c r="B4" s="92"/>
+      <c r="C4" s="92"/>
+      <c r="D4" s="92"/>
+      <c r="E4" s="92"/>
+      <c r="F4" s="92"/>
+      <c r="G4" s="92"/>
+      <c r="H4" s="92"/>
+      <c r="I4" s="92"/>
+      <c r="J4" s="92"/>
+      <c r="K4" s="92"/>
+      <c r="L4" s="92"/>
+      <c r="M4" s="92"/>
+      <c r="N4" s="92"/>
+      <c r="O4" s="92"/>
+      <c r="P4" s="92"/>
+      <c r="Q4" s="92"/>
+      <c r="R4" s="92"/>
+      <c r="S4" s="92"/>
+      <c r="T4" s="92"/>
+      <c r="U4" s="92"/>
+      <c r="V4" s="30" t="s">
+        <v>80</v>
+      </c>
+      <c r="W4" s="30" t="s">
+        <v>81</v>
+      </c>
+      <c r="X4" s="30" t="s">
+        <v>82</v>
+      </c>
+      <c r="Y4" s="30" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A5" s="91"/>
+      <c r="B5" s="31" t="s">
+        <v>84</v>
+      </c>
+      <c r="C5" s="31" t="s">
+        <v>84</v>
+      </c>
+      <c r="D5" s="31" t="s">
+        <v>84</v>
+      </c>
+      <c r="E5" s="92"/>
+      <c r="F5" s="92"/>
+      <c r="G5" s="31" t="s">
+        <v>85</v>
+      </c>
+      <c r="H5" s="31" t="s">
+        <v>85</v>
+      </c>
+      <c r="I5" s="31" t="s">
+        <v>85</v>
+      </c>
+      <c r="J5" s="92"/>
+      <c r="K5" s="31" t="s">
+        <v>86</v>
+      </c>
+      <c r="L5" s="31" t="s">
+        <v>86</v>
+      </c>
+      <c r="M5" s="31" t="s">
+        <v>86</v>
+      </c>
+      <c r="N5" s="92"/>
+      <c r="O5" s="31" t="s">
+        <v>87</v>
+      </c>
+      <c r="P5" s="31" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q5" s="31" t="s">
+        <v>87</v>
+      </c>
+      <c r="R5" s="92"/>
+      <c r="S5" s="92"/>
+      <c r="T5" s="92"/>
+      <c r="U5" s="92"/>
+      <c r="V5" s="92">
+        <v>1</v>
+      </c>
+      <c r="W5" s="92">
+        <v>39600</v>
+      </c>
+      <c r="X5" s="92">
+        <v>39352</v>
+      </c>
+      <c r="Y5" s="93">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A6" s="91"/>
+      <c r="B6" s="30" t="s">
+        <v>88</v>
+      </c>
+      <c r="C6" s="30" t="s">
+        <v>89</v>
+      </c>
+      <c r="D6" s="30" t="s">
+        <v>90</v>
+      </c>
+      <c r="E6" s="92"/>
+      <c r="F6" s="92"/>
+      <c r="G6" s="30" t="s">
+        <v>88</v>
+      </c>
+      <c r="H6" s="30" t="s">
+        <v>89</v>
+      </c>
+      <c r="I6" s="30" t="s">
+        <v>90</v>
+      </c>
+      <c r="J6" s="92"/>
+      <c r="K6" s="30" t="s">
+        <v>88</v>
+      </c>
+      <c r="L6" s="30" t="s">
+        <v>89</v>
+      </c>
+      <c r="M6" s="30" t="s">
+        <v>90</v>
+      </c>
+      <c r="N6" s="92"/>
+      <c r="O6" s="30" t="s">
+        <v>88</v>
+      </c>
+      <c r="P6" s="30" t="s">
+        <v>89</v>
+      </c>
+      <c r="Q6" s="30" t="s">
+        <v>90</v>
+      </c>
+      <c r="R6" s="92"/>
+      <c r="S6" s="30" t="s">
         <v>91</v>
       </c>
-      <c r="C3" s="30" t="s">
-        <v>91</v>
-      </c>
-      <c r="D3" s="103">
-        <v>114</v>
-      </c>
-      <c r="E3" s="103">
-        <v>114</v>
-      </c>
-      <c r="F3" s="103">
-        <v>114</v>
-      </c>
-      <c r="G3" s="103">
-        <v>114</v>
-      </c>
-      <c r="H3" s="103"/>
-      <c r="I3" s="103"/>
-      <c r="J3" s="103"/>
-      <c r="K3" s="103"/>
-      <c r="L3" s="103"/>
-      <c r="M3" s="103"/>
-      <c r="N3" s="103"/>
-      <c r="O3" s="103"/>
-      <c r="P3" s="103"/>
-      <c r="Q3" s="103"/>
-      <c r="R3" s="103"/>
-      <c r="S3" s="103"/>
-      <c r="T3" s="103"/>
-      <c r="U3" s="103"/>
-      <c r="V3" s="30" t="s">
-        <v>92</v>
-      </c>
-      <c r="W3" s="30" t="s">
-        <v>92</v>
-      </c>
-      <c r="X3" s="30" t="s">
-        <v>92</v>
-      </c>
-      <c r="Y3" s="30" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="4" ht="24" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A4" s="102"/>
-      <c r="B4" s="103"/>
-      <c r="C4" s="103"/>
-      <c r="D4" s="103"/>
-      <c r="E4" s="103"/>
-      <c r="F4" s="103"/>
-      <c r="G4" s="103"/>
-      <c r="H4" s="103"/>
-      <c r="I4" s="103"/>
-      <c r="J4" s="103"/>
-      <c r="K4" s="103"/>
-      <c r="L4" s="103"/>
-      <c r="M4" s="103"/>
-      <c r="N4" s="103"/>
-      <c r="O4" s="103"/>
-      <c r="P4" s="103"/>
-      <c r="Q4" s="103"/>
-      <c r="R4" s="103"/>
-      <c r="S4" s="103"/>
-      <c r="T4" s="103"/>
-      <c r="U4" s="103"/>
-      <c r="V4" s="30" t="s">
-        <v>93</v>
-      </c>
-      <c r="W4" s="30" t="s">
-        <v>94</v>
-      </c>
-      <c r="X4" s="30" t="s">
-        <v>95</v>
-      </c>
-      <c r="Y4" s="30" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="5" ht="24" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A5" s="102"/>
-      <c r="B5" s="31" t="s">
-        <v>97</v>
-      </c>
-      <c r="C5" s="31" t="s">
-        <v>97</v>
-      </c>
-      <c r="D5" s="31" t="s">
-        <v>97</v>
-      </c>
-      <c r="E5" s="103"/>
-      <c r="F5" s="103"/>
-      <c r="G5" s="31" t="s">
-        <v>98</v>
-      </c>
-      <c r="H5" s="31" t="s">
-        <v>98</v>
-      </c>
-      <c r="I5" s="31" t="s">
-        <v>98</v>
-      </c>
-      <c r="J5" s="103"/>
-      <c r="K5" s="31" t="s">
-        <v>99</v>
-      </c>
-      <c r="L5" s="31" t="s">
-        <v>99</v>
-      </c>
-      <c r="M5" s="31" t="s">
-        <v>99</v>
-      </c>
-      <c r="N5" s="103"/>
-      <c r="O5" s="31" t="s">
-        <v>100</v>
-      </c>
-      <c r="P5" s="31" t="s">
-        <v>100</v>
-      </c>
-      <c r="Q5" s="31" t="s">
-        <v>100</v>
-      </c>
-      <c r="R5" s="103"/>
-      <c r="S5" s="103"/>
-      <c r="T5" s="103"/>
-      <c r="U5" s="103"/>
-      <c r="V5" s="103">
-        <v>1</v>
-      </c>
-      <c r="W5" s="103">
-        <v>39600</v>
-      </c>
-      <c r="X5" s="103">
-        <v>39352</v>
-      </c>
-      <c r="Y5" s="104">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="6" ht="24" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A6" s="102"/>
-      <c r="B6" s="30" t="s">
-        <v>101</v>
-      </c>
-      <c r="C6" s="30" t="s">
-        <v>102</v>
-      </c>
-      <c r="D6" s="30" t="s">
-        <v>103</v>
-      </c>
-      <c r="E6" s="103"/>
-      <c r="F6" s="103"/>
-      <c r="G6" s="30" t="s">
-        <v>101</v>
-      </c>
-      <c r="H6" s="30" t="s">
-        <v>102</v>
-      </c>
-      <c r="I6" s="30" t="s">
-        <v>103</v>
-      </c>
-      <c r="J6" s="103"/>
-      <c r="K6" s="30" t="s">
-        <v>101</v>
-      </c>
-      <c r="L6" s="30" t="s">
-        <v>102</v>
-      </c>
-      <c r="M6" s="30" t="s">
-        <v>103</v>
-      </c>
-      <c r="N6" s="103"/>
-      <c r="O6" s="30" t="s">
-        <v>101</v>
-      </c>
-      <c r="P6" s="30" t="s">
-        <v>102</v>
-      </c>
-      <c r="Q6" s="30" t="s">
-        <v>103</v>
-      </c>
-      <c r="R6" s="103"/>
-      <c r="S6" s="30" t="s">
-        <v>104</v>
-      </c>
-      <c r="T6" s="103"/>
-      <c r="U6" s="103"/>
-      <c r="V6" s="103">
+      <c r="T6" s="92"/>
+      <c r="U6" s="92"/>
+      <c r="V6" s="92">
         <v>2</v>
       </c>
-      <c r="W6" s="103">
+      <c r="W6" s="92">
         <v>39400</v>
       </c>
-      <c r="X6" s="103">
+      <c r="X6" s="92">
         <v>38360</v>
       </c>
-      <c r="Y6" s="104">
+      <c r="Y6" s="93">
         <v>1040</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A7" s="97"/>
-      <c r="B7" s="105">
+      <c r="A7" s="94"/>
+      <c r="B7" s="95">
         <v>46097</v>
       </c>
       <c r="C7" s="61">
@@ -30803,7 +30251,7 @@
       </c>
       <c r="E7" s="62"/>
       <c r="F7" s="62"/>
-      <c r="G7" s="105">
+      <c r="G7" s="95">
         <v>46107</v>
       </c>
       <c r="H7" s="61">
@@ -30813,20 +30261,20 @@
         <v>43600</v>
       </c>
       <c r="J7" s="62"/>
-      <c r="K7" s="105"/>
+      <c r="K7" s="95"/>
       <c r="L7" s="62"/>
       <c r="M7" s="62"/>
       <c r="N7" s="62"/>
-      <c r="O7" s="105"/>
+      <c r="O7" s="95"/>
       <c r="P7" s="62"/>
       <c r="Q7" s="62"/>
       <c r="R7" s="62"/>
       <c r="S7" s="62" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="T7" s="62"/>
       <c r="U7" s="62"/>
-      <c r="V7" s="106">
+      <c r="V7" s="96">
         <v>3</v>
       </c>
       <c r="W7" s="61">
@@ -30835,13 +30283,13 @@
       <c r="X7" s="61">
         <v>41088</v>
       </c>
-      <c r="Y7" s="107">
+      <c r="Y7" s="97">
         <v>-1088</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A8" s="93"/>
-      <c r="B8" s="108">
+      <c r="A8" s="98"/>
+      <c r="B8" s="99">
         <v>46096</v>
       </c>
       <c r="C8" s="71">
@@ -30850,9 +30298,9 @@
       <c r="D8" s="71">
         <v>44000</v>
       </c>
-      <c r="E8" s="95"/>
-      <c r="F8" s="95"/>
-      <c r="G8" s="108">
+      <c r="E8" s="100"/>
+      <c r="F8" s="100"/>
+      <c r="G8" s="99">
         <v>46107</v>
       </c>
       <c r="H8" s="71">
@@ -30861,21 +30309,21 @@
       <c r="I8" s="71">
         <v>43640</v>
       </c>
-      <c r="J8" s="95"/>
-      <c r="K8" s="108"/>
-      <c r="L8" s="95"/>
-      <c r="M8" s="95"/>
-      <c r="N8" s="95"/>
-      <c r="O8" s="108"/>
-      <c r="P8" s="95"/>
-      <c r="Q8" s="95"/>
-      <c r="R8" s="95"/>
+      <c r="J8" s="100"/>
+      <c r="K8" s="99"/>
+      <c r="L8" s="100"/>
+      <c r="M8" s="100"/>
+      <c r="N8" s="100"/>
+      <c r="O8" s="99"/>
+      <c r="P8" s="100"/>
+      <c r="Q8" s="100"/>
+      <c r="R8" s="100"/>
       <c r="S8" s="71">
         <v>168000</v>
       </c>
-      <c r="T8" s="95"/>
-      <c r="U8" s="95"/>
-      <c r="V8" s="109">
+      <c r="T8" s="100"/>
+      <c r="U8" s="100"/>
+      <c r="V8" s="101">
         <v>4</v>
       </c>
       <c r="W8" s="71">
@@ -30884,13 +30332,13 @@
       <c r="X8" s="71">
         <v>38784</v>
       </c>
-      <c r="Y8" s="110">
+      <c r="Y8" s="102">
         <v>1216</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A9" s="97"/>
-      <c r="B9" s="105">
+      <c r="A9" s="94"/>
+      <c r="B9" s="95">
         <v>46096</v>
       </c>
       <c r="C9" s="61">
@@ -30901,22 +30349,22 @@
       </c>
       <c r="E9" s="62"/>
       <c r="F9" s="62"/>
-      <c r="G9" s="105"/>
+      <c r="G9" s="95"/>
       <c r="H9" s="62"/>
       <c r="I9" s="62"/>
       <c r="J9" s="62"/>
-      <c r="K9" s="105"/>
+      <c r="K9" s="95"/>
       <c r="L9" s="62"/>
       <c r="M9" s="62"/>
       <c r="N9" s="62"/>
-      <c r="O9" s="105"/>
+      <c r="O9" s="95"/>
       <c r="P9" s="62"/>
       <c r="Q9" s="62"/>
       <c r="R9" s="62"/>
       <c r="S9" s="62"/>
       <c r="T9" s="62"/>
       <c r="U9" s="62"/>
-      <c r="V9" s="106">
+      <c r="V9" s="96">
         <v>5</v>
       </c>
       <c r="W9" s="61">
@@ -30925,13 +30373,13 @@
       <c r="X9" s="61">
         <v>39680</v>
       </c>
-      <c r="Y9" s="107">
+      <c r="Y9" s="97">
         <v>720</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A10" s="93"/>
-      <c r="B10" s="108">
+      <c r="A10" s="98"/>
+      <c r="B10" s="99">
         <v>46096</v>
       </c>
       <c r="C10" s="71">
@@ -30940,26 +30388,26 @@
       <c r="D10" s="71">
         <v>43860</v>
       </c>
-      <c r="E10" s="95"/>
-      <c r="F10" s="95"/>
-      <c r="G10" s="108"/>
-      <c r="H10" s="95"/>
-      <c r="I10" s="95"/>
-      <c r="J10" s="95"/>
-      <c r="K10" s="108"/>
-      <c r="L10" s="95"/>
-      <c r="M10" s="95"/>
-      <c r="N10" s="95"/>
-      <c r="O10" s="108"/>
-      <c r="P10" s="95"/>
-      <c r="Q10" s="95"/>
-      <c r="R10" s="95"/>
-      <c r="S10" s="111" t="s">
-        <v>106</v>
-      </c>
-      <c r="T10" s="95"/>
-      <c r="U10" s="95"/>
-      <c r="V10" s="109">
+      <c r="E10" s="100"/>
+      <c r="F10" s="100"/>
+      <c r="G10" s="99"/>
+      <c r="H10" s="100"/>
+      <c r="I10" s="100"/>
+      <c r="J10" s="100"/>
+      <c r="K10" s="99"/>
+      <c r="L10" s="100"/>
+      <c r="M10" s="100"/>
+      <c r="N10" s="100"/>
+      <c r="O10" s="99"/>
+      <c r="P10" s="100"/>
+      <c r="Q10" s="100"/>
+      <c r="R10" s="100"/>
+      <c r="S10" s="103" t="s">
+        <v>93</v>
+      </c>
+      <c r="T10" s="100"/>
+      <c r="U10" s="100"/>
+      <c r="V10" s="101">
         <v>6</v>
       </c>
       <c r="W10" s="71">
@@ -30968,35 +30416,35 @@
       <c r="X10" s="71">
         <v>38230</v>
       </c>
-      <c r="Y10" s="110">
+      <c r="Y10" s="102">
         <v>1980</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A11" s="97"/>
-      <c r="B11" s="105"/>
+      <c r="A11" s="94"/>
+      <c r="B11" s="95"/>
       <c r="C11" s="62"/>
       <c r="D11" s="62"/>
       <c r="E11" s="62"/>
       <c r="F11" s="62"/>
-      <c r="G11" s="105"/>
+      <c r="G11" s="95"/>
       <c r="H11" s="62"/>
       <c r="I11" s="62"/>
       <c r="J11" s="62"/>
-      <c r="K11" s="105"/>
+      <c r="K11" s="95"/>
       <c r="L11" s="62"/>
       <c r="M11" s="62"/>
       <c r="N11" s="62"/>
-      <c r="O11" s="105"/>
+      <c r="O11" s="95"/>
       <c r="P11" s="62"/>
       <c r="Q11" s="62"/>
       <c r="R11" s="62"/>
-      <c r="S11" s="111" t="s">
-        <v>107</v>
+      <c r="S11" s="103" t="s">
+        <v>94</v>
       </c>
       <c r="T11" s="62"/>
       <c r="U11" s="62"/>
-      <c r="V11" s="106">
+      <c r="V11" s="96">
         <v>7</v>
       </c>
       <c r="W11" s="61">
@@ -31005,36 +30453,36 @@
       <c r="X11" s="61">
         <v>48400</v>
       </c>
-      <c r="Y11" s="112">
+      <c r="Y11" s="104">
         <v>1904</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A12" s="93"/>
-      <c r="B12" s="108"/>
-      <c r="C12" s="95"/>
-      <c r="D12" s="95"/>
-      <c r="E12" s="95"/>
-      <c r="F12" s="95"/>
-      <c r="G12" s="108"/>
-      <c r="H12" s="95"/>
-      <c r="I12" s="95"/>
-      <c r="J12" s="95"/>
-      <c r="K12" s="108"/>
-      <c r="L12" s="95"/>
-      <c r="M12" s="95"/>
-      <c r="N12" s="95"/>
-      <c r="O12" s="108"/>
-      <c r="P12" s="95"/>
-      <c r="Q12" s="95"/>
-      <c r="R12" s="95"/>
-      <c r="S12" s="109">
+      <c r="A12" s="98"/>
+      <c r="B12" s="99"/>
+      <c r="C12" s="100"/>
+      <c r="D12" s="100"/>
+      <c r="E12" s="100"/>
+      <c r="F12" s="100"/>
+      <c r="G12" s="99"/>
+      <c r="H12" s="100"/>
+      <c r="I12" s="100"/>
+      <c r="J12" s="100"/>
+      <c r="K12" s="99"/>
+      <c r="L12" s="100"/>
+      <c r="M12" s="100"/>
+      <c r="N12" s="100"/>
+      <c r="O12" s="99"/>
+      <c r="P12" s="100"/>
+      <c r="Q12" s="100"/>
+      <c r="R12" s="100"/>
+      <c r="S12" s="101">
         <f>+D37+I37+M37+Q37</f>
         <v>261000</v>
       </c>
-      <c r="T12" s="95"/>
-      <c r="U12" s="95"/>
-      <c r="V12" s="109">
+      <c r="T12" s="100"/>
+      <c r="U12" s="100"/>
+      <c r="V12" s="101">
         <v>8</v>
       </c>
       <c r="W12" s="71">
@@ -31043,33 +30491,33 @@
       <c r="X12" s="71">
         <v>47648</v>
       </c>
-      <c r="Y12" s="113">
+      <c r="Y12" s="105">
         <v>138</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A13" s="97"/>
-      <c r="B13" s="105"/>
+      <c r="A13" s="94"/>
+      <c r="B13" s="95"/>
       <c r="C13" s="62"/>
       <c r="D13" s="62"/>
       <c r="E13" s="62"/>
       <c r="F13" s="62"/>
-      <c r="G13" s="105"/>
+      <c r="G13" s="95"/>
       <c r="H13" s="62"/>
       <c r="I13" s="62"/>
       <c r="J13" s="62"/>
-      <c r="K13" s="105"/>
+      <c r="K13" s="95"/>
       <c r="L13" s="62"/>
       <c r="M13" s="62"/>
       <c r="N13" s="62"/>
-      <c r="O13" s="105"/>
+      <c r="O13" s="95"/>
       <c r="P13" s="62"/>
       <c r="Q13" s="62"/>
       <c r="R13" s="62"/>
       <c r="S13" s="62"/>
       <c r="T13" s="62"/>
       <c r="U13" s="62"/>
-      <c r="V13" s="106">
+      <c r="V13" s="96">
         <v>9</v>
       </c>
       <c r="W13" s="61">
@@ -31078,35 +30526,35 @@
       <c r="X13" s="61">
         <v>46120</v>
       </c>
-      <c r="Y13" s="112">
+      <c r="Y13" s="104">
         <v>1980</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A14" s="93"/>
-      <c r="B14" s="108"/>
-      <c r="C14" s="95"/>
-      <c r="D14" s="95"/>
-      <c r="E14" s="95"/>
-      <c r="F14" s="95"/>
-      <c r="G14" s="108"/>
-      <c r="H14" s="95"/>
-      <c r="I14" s="95"/>
-      <c r="J14" s="95"/>
-      <c r="K14" s="108"/>
-      <c r="L14" s="95"/>
-      <c r="M14" s="95"/>
-      <c r="N14" s="95"/>
-      <c r="O14" s="108"/>
-      <c r="P14" s="95"/>
-      <c r="Q14" s="95"/>
-      <c r="R14" s="95"/>
-      <c r="S14" s="111" t="s">
-        <v>108</v>
-      </c>
-      <c r="T14" s="95"/>
-      <c r="U14" s="95"/>
-      <c r="V14" s="109">
+      <c r="A14" s="98"/>
+      <c r="B14" s="99"/>
+      <c r="C14" s="100"/>
+      <c r="D14" s="100"/>
+      <c r="E14" s="100"/>
+      <c r="F14" s="100"/>
+      <c r="G14" s="99"/>
+      <c r="H14" s="100"/>
+      <c r="I14" s="100"/>
+      <c r="J14" s="100"/>
+      <c r="K14" s="99"/>
+      <c r="L14" s="100"/>
+      <c r="M14" s="100"/>
+      <c r="N14" s="100"/>
+      <c r="O14" s="99"/>
+      <c r="P14" s="100"/>
+      <c r="Q14" s="100"/>
+      <c r="R14" s="100"/>
+      <c r="S14" s="103" t="s">
+        <v>95</v>
+      </c>
+      <c r="T14" s="100"/>
+      <c r="U14" s="100"/>
+      <c r="V14" s="101">
         <v>10</v>
       </c>
       <c r="W14" s="71">
@@ -31115,35 +30563,35 @@
       <c r="X14" s="71">
         <v>47152</v>
       </c>
-      <c r="Y14" s="113">
+      <c r="Y14" s="105">
         <v>948</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A15" s="97"/>
-      <c r="B15" s="105"/>
+      <c r="A15" s="94"/>
+      <c r="B15" s="95"/>
       <c r="C15" s="62"/>
       <c r="D15" s="62"/>
       <c r="E15" s="62"/>
       <c r="F15" s="62"/>
-      <c r="G15" s="105"/>
+      <c r="G15" s="95"/>
       <c r="H15" s="62"/>
       <c r="I15" s="62"/>
       <c r="J15" s="62"/>
-      <c r="K15" s="105"/>
+      <c r="K15" s="95"/>
       <c r="L15" s="62"/>
       <c r="M15" s="62"/>
       <c r="N15" s="62"/>
-      <c r="O15" s="105"/>
+      <c r="O15" s="95"/>
       <c r="P15" s="62"/>
       <c r="Q15" s="62"/>
       <c r="R15" s="62"/>
       <c r="S15" s="62" t="s">
-        <v>109</v>
+        <v>96</v>
       </c>
       <c r="T15" s="62"/>
       <c r="U15" s="62"/>
-      <c r="V15" s="106">
+      <c r="V15" s="96">
         <v>11</v>
       </c>
       <c r="W15" s="61">
@@ -31152,33 +30600,33 @@
       <c r="X15" s="61">
         <v>43456</v>
       </c>
-      <c r="Y15" s="112">
+      <c r="Y15" s="104">
         <v>4644</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A16" s="93"/>
-      <c r="B16" s="108"/>
-      <c r="C16" s="95"/>
-      <c r="D16" s="95"/>
-      <c r="E16" s="95"/>
-      <c r="F16" s="95"/>
-      <c r="G16" s="108"/>
-      <c r="H16" s="95"/>
-      <c r="I16" s="95"/>
-      <c r="J16" s="95"/>
-      <c r="K16" s="108"/>
-      <c r="L16" s="95"/>
-      <c r="M16" s="95"/>
-      <c r="N16" s="95"/>
-      <c r="O16" s="108"/>
-      <c r="P16" s="95"/>
-      <c r="Q16" s="95"/>
-      <c r="R16" s="95"/>
-      <c r="S16" s="95"/>
-      <c r="T16" s="95"/>
-      <c r="U16" s="95"/>
-      <c r="V16" s="109">
+      <c r="A16" s="98"/>
+      <c r="B16" s="99"/>
+      <c r="C16" s="100"/>
+      <c r="D16" s="100"/>
+      <c r="E16" s="100"/>
+      <c r="F16" s="100"/>
+      <c r="G16" s="99"/>
+      <c r="H16" s="100"/>
+      <c r="I16" s="100"/>
+      <c r="J16" s="100"/>
+      <c r="K16" s="99"/>
+      <c r="L16" s="100"/>
+      <c r="M16" s="100"/>
+      <c r="N16" s="100"/>
+      <c r="O16" s="99"/>
+      <c r="P16" s="100"/>
+      <c r="Q16" s="100"/>
+      <c r="R16" s="100"/>
+      <c r="S16" s="100"/>
+      <c r="T16" s="100"/>
+      <c r="U16" s="100"/>
+      <c r="V16" s="101">
         <v>12</v>
       </c>
       <c r="W16" s="71">
@@ -31187,218 +30635,218 @@
       <c r="X16" s="71">
         <v>49064</v>
       </c>
-      <c r="Y16" s="113">
+      <c r="Y16" s="105">
         <v>336</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A17" s="97"/>
-      <c r="B17" s="105"/>
+      <c r="A17" s="94"/>
+      <c r="B17" s="95"/>
       <c r="C17" s="62"/>
       <c r="D17" s="62"/>
       <c r="E17" s="62"/>
       <c r="F17" s="62"/>
-      <c r="G17" s="105"/>
+      <c r="G17" s="95"/>
       <c r="H17" s="62"/>
       <c r="I17" s="62"/>
       <c r="J17" s="62"/>
-      <c r="K17" s="105"/>
+      <c r="K17" s="95"/>
       <c r="L17" s="62"/>
       <c r="M17" s="62"/>
       <c r="N17" s="62"/>
-      <c r="O17" s="105"/>
+      <c r="O17" s="95"/>
       <c r="P17" s="62"/>
       <c r="Q17" s="62"/>
       <c r="R17" s="62"/>
       <c r="S17" s="62"/>
       <c r="T17" s="62"/>
       <c r="U17" s="62"/>
-      <c r="V17" s="111" t="s">
-        <v>110</v>
+      <c r="V17" s="103" t="s">
+        <v>97</v>
       </c>
       <c r="W17" s="62" t="s">
-        <v>111</v>
+        <v>98</v>
       </c>
       <c r="X17" s="61">
         <f>SUM(X5:X16)</f>
         <v>517334</v>
       </c>
-      <c r="Y17" s="112">
+      <c r="Y17" s="104">
         <f>SUM(Y5:Y16)</f>
         <v>14102</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A18" s="93"/>
-      <c r="B18" s="108"/>
-      <c r="C18" s="95"/>
-      <c r="D18" s="95"/>
-      <c r="E18" s="95"/>
-      <c r="F18" s="95"/>
-      <c r="G18" s="108"/>
-      <c r="H18" s="95"/>
-      <c r="I18" s="95"/>
-      <c r="J18" s="95"/>
-      <c r="K18" s="108"/>
-      <c r="L18" s="95"/>
-      <c r="M18" s="95"/>
-      <c r="N18" s="95"/>
-      <c r="O18" s="108"/>
-      <c r="P18" s="95"/>
-      <c r="Q18" s="95"/>
-      <c r="R18" s="95"/>
-      <c r="S18" s="111" t="s">
-        <v>112</v>
-      </c>
-      <c r="T18" s="95"/>
-      <c r="U18" s="95"/>
-      <c r="V18" s="111" t="s">
-        <v>113</v>
-      </c>
-      <c r="W18" s="111" t="s">
-        <v>113</v>
-      </c>
-      <c r="X18" s="95"/>
-      <c r="Y18" s="96"/>
+      <c r="A18" s="98"/>
+      <c r="B18" s="99"/>
+      <c r="C18" s="100"/>
+      <c r="D18" s="100"/>
+      <c r="E18" s="100"/>
+      <c r="F18" s="100"/>
+      <c r="G18" s="99"/>
+      <c r="H18" s="100"/>
+      <c r="I18" s="100"/>
+      <c r="J18" s="100"/>
+      <c r="K18" s="99"/>
+      <c r="L18" s="100"/>
+      <c r="M18" s="100"/>
+      <c r="N18" s="100"/>
+      <c r="O18" s="99"/>
+      <c r="P18" s="100"/>
+      <c r="Q18" s="100"/>
+      <c r="R18" s="100"/>
+      <c r="S18" s="103" t="s">
+        <v>99</v>
+      </c>
+      <c r="T18" s="100"/>
+      <c r="U18" s="100"/>
+      <c r="V18" s="103" t="s">
+        <v>100</v>
+      </c>
+      <c r="W18" s="103" t="s">
+        <v>100</v>
+      </c>
+      <c r="X18" s="100"/>
+      <c r="Y18" s="106"/>
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A19" s="97"/>
-      <c r="B19" s="105"/>
+      <c r="A19" s="94"/>
+      <c r="B19" s="95"/>
       <c r="C19" s="62"/>
       <c r="D19" s="62"/>
       <c r="E19" s="62"/>
       <c r="F19" s="62"/>
-      <c r="G19" s="105"/>
+      <c r="G19" s="95"/>
       <c r="H19" s="62"/>
       <c r="I19" s="62"/>
       <c r="J19" s="62"/>
-      <c r="K19" s="105"/>
+      <c r="K19" s="95"/>
       <c r="L19" s="62"/>
       <c r="M19" s="62"/>
       <c r="N19" s="62"/>
-      <c r="O19" s="105"/>
+      <c r="O19" s="95"/>
       <c r="P19" s="62"/>
       <c r="Q19" s="62"/>
       <c r="R19" s="62"/>
-      <c r="S19" s="106">
+      <c r="S19" s="96">
         <f>+S8+S12-S16</f>
         <v>429000</v>
       </c>
       <c r="T19" s="62"/>
       <c r="U19" s="62"/>
-      <c r="V19" s="111" t="s">
-        <v>114</v>
-      </c>
-      <c r="W19" s="111" t="s">
-        <v>114</v>
+      <c r="V19" s="103" t="s">
+        <v>101</v>
+      </c>
+      <c r="W19" s="103" t="s">
+        <v>101</v>
       </c>
       <c r="X19" s="61">
         <v>168000</v>
       </c>
-      <c r="Y19" s="98"/>
+      <c r="Y19" s="107"/>
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A20" s="93"/>
-      <c r="B20" s="108"/>
-      <c r="C20" s="95"/>
-      <c r="D20" s="95"/>
-      <c r="E20" s="95"/>
-      <c r="F20" s="95"/>
-      <c r="G20" s="108"/>
-      <c r="H20" s="95"/>
-      <c r="I20" s="95"/>
-      <c r="J20" s="95"/>
-      <c r="K20" s="108"/>
-      <c r="L20" s="95"/>
-      <c r="M20" s="95"/>
-      <c r="N20" s="95"/>
-      <c r="O20" s="108"/>
-      <c r="P20" s="95"/>
-      <c r="Q20" s="95"/>
-      <c r="R20" s="95"/>
-      <c r="S20" s="95"/>
-      <c r="T20" s="95"/>
-      <c r="U20" s="95"/>
-      <c r="V20" s="111" t="s">
-        <v>115</v>
-      </c>
-      <c r="W20" s="111" t="s">
-        <v>115</v>
+      <c r="A20" s="98"/>
+      <c r="B20" s="99"/>
+      <c r="C20" s="100"/>
+      <c r="D20" s="100"/>
+      <c r="E20" s="100"/>
+      <c r="F20" s="100"/>
+      <c r="G20" s="99"/>
+      <c r="H20" s="100"/>
+      <c r="I20" s="100"/>
+      <c r="J20" s="100"/>
+      <c r="K20" s="99"/>
+      <c r="L20" s="100"/>
+      <c r="M20" s="100"/>
+      <c r="N20" s="100"/>
+      <c r="O20" s="99"/>
+      <c r="P20" s="100"/>
+      <c r="Q20" s="100"/>
+      <c r="R20" s="100"/>
+      <c r="S20" s="100"/>
+      <c r="T20" s="100"/>
+      <c r="U20" s="100"/>
+      <c r="V20" s="103" t="s">
+        <v>102</v>
+      </c>
+      <c r="W20" s="103" t="s">
+        <v>102</v>
       </c>
       <c r="X20" s="71">
         <v>2142600</v>
       </c>
-      <c r="Y20" s="96"/>
+      <c r="Y20" s="106"/>
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A21" s="97"/>
-      <c r="B21" s="105"/>
+      <c r="A21" s="94"/>
+      <c r="B21" s="95"/>
       <c r="C21" s="62"/>
       <c r="D21" s="62"/>
       <c r="E21" s="62"/>
       <c r="F21" s="62"/>
-      <c r="G21" s="105"/>
+      <c r="G21" s="95"/>
       <c r="H21" s="62"/>
       <c r="I21" s="62"/>
       <c r="J21" s="62"/>
-      <c r="K21" s="105"/>
+      <c r="K21" s="95"/>
       <c r="L21" s="62"/>
       <c r="M21" s="62"/>
       <c r="N21" s="62"/>
-      <c r="O21" s="105"/>
+      <c r="O21" s="95"/>
       <c r="P21" s="62"/>
       <c r="Q21" s="62"/>
       <c r="R21" s="62"/>
       <c r="S21" s="62"/>
       <c r="T21" s="62"/>
       <c r="U21" s="62"/>
-      <c r="V21" s="111" t="s">
-        <v>116</v>
-      </c>
-      <c r="W21" s="111" t="s">
-        <v>116</v>
+      <c r="V21" s="103" t="s">
+        <v>103</v>
+      </c>
+      <c r="W21" s="103" t="s">
+        <v>103</v>
       </c>
       <c r="X21" s="61">
         <v>168000</v>
       </c>
-      <c r="Y21" s="98"/>
+      <c r="Y21" s="107"/>
     </row>
     <row r="22" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A22" s="93"/>
-      <c r="B22" s="108"/>
-      <c r="C22" s="95"/>
-      <c r="D22" s="95"/>
-      <c r="E22" s="95"/>
-      <c r="F22" s="95"/>
-      <c r="G22" s="108"/>
-      <c r="H22" s="95"/>
-      <c r="I22" s="95"/>
-      <c r="J22" s="95"/>
-      <c r="K22" s="108"/>
-      <c r="L22" s="95"/>
-      <c r="M22" s="95"/>
-      <c r="N22" s="95"/>
-      <c r="O22" s="108"/>
-      <c r="P22" s="95"/>
-      <c r="Q22" s="95"/>
-      <c r="R22" s="95"/>
-      <c r="S22" s="95"/>
-      <c r="T22" s="95"/>
-      <c r="U22" s="95"/>
-      <c r="V22" s="111" t="s">
-        <v>117</v>
-      </c>
-      <c r="W22" s="111" t="s">
-        <v>117</v>
+      <c r="A22" s="98"/>
+      <c r="B22" s="99"/>
+      <c r="C22" s="100"/>
+      <c r="D22" s="100"/>
+      <c r="E22" s="100"/>
+      <c r="F22" s="100"/>
+      <c r="G22" s="99"/>
+      <c r="H22" s="100"/>
+      <c r="I22" s="100"/>
+      <c r="J22" s="100"/>
+      <c r="K22" s="99"/>
+      <c r="L22" s="100"/>
+      <c r="M22" s="100"/>
+      <c r="N22" s="100"/>
+      <c r="O22" s="99"/>
+      <c r="P22" s="100"/>
+      <c r="Q22" s="100"/>
+      <c r="R22" s="100"/>
+      <c r="S22" s="100"/>
+      <c r="T22" s="100"/>
+      <c r="U22" s="100"/>
+      <c r="V22" s="103" t="s">
+        <v>104</v>
+      </c>
+      <c r="W22" s="103" t="s">
+        <v>104</v>
       </c>
       <c r="X22" s="71">
         <f>X19+X20-X21</f>
         <v>2142600</v>
       </c>
-      <c r="Y22" s="96"/>
+      <c r="Y22" s="106"/>
     </row>
     <row r="23" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A23" s="97"/>
+      <c r="A23" s="94"/>
       <c r="B23" s="62"/>
       <c r="C23" s="62"/>
       <c r="D23" s="62"/>
@@ -31422,37 +30870,37 @@
       <c r="V23" s="62"/>
       <c r="W23" s="62"/>
       <c r="X23" s="62"/>
-      <c r="Y23" s="98"/>
+      <c r="Y23" s="107"/>
     </row>
     <row r="24" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A24" s="93"/>
-      <c r="B24" s="95"/>
-      <c r="C24" s="95"/>
-      <c r="D24" s="95"/>
-      <c r="E24" s="95"/>
-      <c r="F24" s="95"/>
-      <c r="G24" s="95"/>
-      <c r="H24" s="95"/>
-      <c r="I24" s="95"/>
-      <c r="J24" s="95"/>
-      <c r="K24" s="95"/>
-      <c r="L24" s="95"/>
-      <c r="M24" s="95"/>
-      <c r="N24" s="95"/>
-      <c r="O24" s="95"/>
-      <c r="P24" s="95"/>
-      <c r="Q24" s="95"/>
-      <c r="R24" s="95"/>
-      <c r="S24" s="95"/>
-      <c r="T24" s="95"/>
-      <c r="U24" s="95"/>
-      <c r="V24" s="95"/>
-      <c r="W24" s="95"/>
-      <c r="X24" s="95"/>
-      <c r="Y24" s="96"/>
+      <c r="A24" s="98"/>
+      <c r="B24" s="100"/>
+      <c r="C24" s="100"/>
+      <c r="D24" s="100"/>
+      <c r="E24" s="100"/>
+      <c r="F24" s="100"/>
+      <c r="G24" s="100"/>
+      <c r="H24" s="100"/>
+      <c r="I24" s="100"/>
+      <c r="J24" s="100"/>
+      <c r="K24" s="100"/>
+      <c r="L24" s="100"/>
+      <c r="M24" s="100"/>
+      <c r="N24" s="100"/>
+      <c r="O24" s="100"/>
+      <c r="P24" s="100"/>
+      <c r="Q24" s="100"/>
+      <c r="R24" s="100"/>
+      <c r="S24" s="100"/>
+      <c r="T24" s="100"/>
+      <c r="U24" s="100"/>
+      <c r="V24" s="100"/>
+      <c r="W24" s="100"/>
+      <c r="X24" s="100"/>
+      <c r="Y24" s="106"/>
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A25" s="97"/>
+      <c r="A25" s="94"/>
       <c r="B25" s="62"/>
       <c r="C25" s="62"/>
       <c r="D25" s="62"/>
@@ -31476,37 +30924,37 @@
       <c r="V25" s="62"/>
       <c r="W25" s="62"/>
       <c r="X25" s="62"/>
-      <c r="Y25" s="98"/>
+      <c r="Y25" s="107"/>
     </row>
     <row r="26" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A26" s="93"/>
-      <c r="B26" s="95"/>
-      <c r="C26" s="95"/>
-      <c r="D26" s="95"/>
-      <c r="E26" s="95"/>
-      <c r="F26" s="95"/>
-      <c r="G26" s="95"/>
-      <c r="H26" s="95"/>
-      <c r="I26" s="95"/>
-      <c r="J26" s="95"/>
-      <c r="K26" s="95"/>
-      <c r="L26" s="95"/>
-      <c r="M26" s="95"/>
-      <c r="N26" s="95"/>
-      <c r="O26" s="95"/>
-      <c r="P26" s="95"/>
-      <c r="Q26" s="95"/>
-      <c r="R26" s="95"/>
-      <c r="S26" s="95"/>
-      <c r="T26" s="95"/>
-      <c r="U26" s="95"/>
-      <c r="V26" s="95"/>
-      <c r="W26" s="95"/>
-      <c r="X26" s="95"/>
-      <c r="Y26" s="96"/>
+      <c r="A26" s="98"/>
+      <c r="B26" s="100"/>
+      <c r="C26" s="100"/>
+      <c r="D26" s="100"/>
+      <c r="E26" s="100"/>
+      <c r="F26" s="100"/>
+      <c r="G26" s="100"/>
+      <c r="H26" s="100"/>
+      <c r="I26" s="100"/>
+      <c r="J26" s="100"/>
+      <c r="K26" s="100"/>
+      <c r="L26" s="100"/>
+      <c r="M26" s="100"/>
+      <c r="N26" s="100"/>
+      <c r="O26" s="100"/>
+      <c r="P26" s="100"/>
+      <c r="Q26" s="100"/>
+      <c r="R26" s="100"/>
+      <c r="S26" s="100"/>
+      <c r="T26" s="100"/>
+      <c r="U26" s="100"/>
+      <c r="V26" s="100"/>
+      <c r="W26" s="100"/>
+      <c r="X26" s="100"/>
+      <c r="Y26" s="106"/>
     </row>
     <row r="27" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A27" s="97"/>
+      <c r="A27" s="94"/>
       <c r="B27" s="62"/>
       <c r="C27" s="62"/>
       <c r="D27" s="62"/>
@@ -31530,37 +30978,37 @@
       <c r="V27" s="62"/>
       <c r="W27" s="62"/>
       <c r="X27" s="62"/>
-      <c r="Y27" s="98"/>
+      <c r="Y27" s="107"/>
     </row>
     <row r="28" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A28" s="93"/>
-      <c r="B28" s="95"/>
-      <c r="C28" s="95"/>
-      <c r="D28" s="95"/>
-      <c r="E28" s="95"/>
-      <c r="F28" s="95"/>
-      <c r="G28" s="95"/>
-      <c r="H28" s="95"/>
-      <c r="I28" s="95"/>
-      <c r="J28" s="95"/>
-      <c r="K28" s="95"/>
-      <c r="L28" s="95"/>
-      <c r="M28" s="95"/>
-      <c r="N28" s="95"/>
-      <c r="O28" s="95"/>
-      <c r="P28" s="95"/>
-      <c r="Q28" s="95"/>
-      <c r="R28" s="95"/>
-      <c r="S28" s="95"/>
-      <c r="T28" s="95"/>
-      <c r="U28" s="95"/>
-      <c r="V28" s="95"/>
-      <c r="W28" s="95"/>
-      <c r="X28" s="95"/>
-      <c r="Y28" s="96"/>
+      <c r="A28" s="98"/>
+      <c r="B28" s="100"/>
+      <c r="C28" s="100"/>
+      <c r="D28" s="100"/>
+      <c r="E28" s="100"/>
+      <c r="F28" s="100"/>
+      <c r="G28" s="100"/>
+      <c r="H28" s="100"/>
+      <c r="I28" s="100"/>
+      <c r="J28" s="100"/>
+      <c r="K28" s="100"/>
+      <c r="L28" s="100"/>
+      <c r="M28" s="100"/>
+      <c r="N28" s="100"/>
+      <c r="O28" s="100"/>
+      <c r="P28" s="100"/>
+      <c r="Q28" s="100"/>
+      <c r="R28" s="100"/>
+      <c r="S28" s="100"/>
+      <c r="T28" s="100"/>
+      <c r="U28" s="100"/>
+      <c r="V28" s="100"/>
+      <c r="W28" s="100"/>
+      <c r="X28" s="100"/>
+      <c r="Y28" s="106"/>
     </row>
     <row r="29" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A29" s="97"/>
+      <c r="A29" s="94"/>
       <c r="B29" s="62"/>
       <c r="C29" s="62"/>
       <c r="D29" s="62"/>
@@ -31584,37 +31032,37 @@
       <c r="V29" s="62"/>
       <c r="W29" s="62"/>
       <c r="X29" s="62"/>
-      <c r="Y29" s="98"/>
+      <c r="Y29" s="107"/>
     </row>
     <row r="30" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A30" s="93"/>
-      <c r="B30" s="95"/>
-      <c r="C30" s="95"/>
-      <c r="D30" s="95"/>
-      <c r="E30" s="95"/>
-      <c r="F30" s="95"/>
-      <c r="G30" s="95"/>
-      <c r="H30" s="95"/>
-      <c r="I30" s="95"/>
-      <c r="J30" s="95"/>
-      <c r="K30" s="95"/>
-      <c r="L30" s="95"/>
-      <c r="M30" s="95"/>
-      <c r="N30" s="95"/>
-      <c r="O30" s="95"/>
-      <c r="P30" s="95"/>
-      <c r="Q30" s="95"/>
-      <c r="R30" s="95"/>
-      <c r="S30" s="95"/>
-      <c r="T30" s="95"/>
-      <c r="U30" s="95"/>
-      <c r="V30" s="95"/>
-      <c r="W30" s="95"/>
-      <c r="X30" s="95"/>
-      <c r="Y30" s="96"/>
+      <c r="A30" s="98"/>
+      <c r="B30" s="100"/>
+      <c r="C30" s="100"/>
+      <c r="D30" s="100"/>
+      <c r="E30" s="100"/>
+      <c r="F30" s="100"/>
+      <c r="G30" s="100"/>
+      <c r="H30" s="100"/>
+      <c r="I30" s="100"/>
+      <c r="J30" s="100"/>
+      <c r="K30" s="100"/>
+      <c r="L30" s="100"/>
+      <c r="M30" s="100"/>
+      <c r="N30" s="100"/>
+      <c r="O30" s="100"/>
+      <c r="P30" s="100"/>
+      <c r="Q30" s="100"/>
+      <c r="R30" s="100"/>
+      <c r="S30" s="100"/>
+      <c r="T30" s="100"/>
+      <c r="U30" s="100"/>
+      <c r="V30" s="100"/>
+      <c r="W30" s="100"/>
+      <c r="X30" s="100"/>
+      <c r="Y30" s="106"/>
     </row>
     <row r="31" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A31" s="97"/>
+      <c r="A31" s="94"/>
       <c r="B31" s="62"/>
       <c r="C31" s="62"/>
       <c r="D31" s="62"/>
@@ -31638,37 +31086,37 @@
       <c r="V31" s="62"/>
       <c r="W31" s="62"/>
       <c r="X31" s="62"/>
-      <c r="Y31" s="98"/>
+      <c r="Y31" s="107"/>
     </row>
     <row r="32" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A32" s="93"/>
-      <c r="B32" s="95"/>
-      <c r="C32" s="95"/>
-      <c r="D32" s="95"/>
-      <c r="E32" s="95"/>
-      <c r="F32" s="95"/>
-      <c r="G32" s="95"/>
-      <c r="H32" s="95"/>
-      <c r="I32" s="95"/>
-      <c r="J32" s="95"/>
-      <c r="K32" s="95"/>
-      <c r="L32" s="95"/>
-      <c r="M32" s="95"/>
-      <c r="N32" s="95"/>
-      <c r="O32" s="95"/>
-      <c r="P32" s="95"/>
-      <c r="Q32" s="95"/>
-      <c r="R32" s="95"/>
-      <c r="S32" s="95"/>
-      <c r="T32" s="95"/>
-      <c r="U32" s="95"/>
-      <c r="V32" s="95"/>
-      <c r="W32" s="95"/>
-      <c r="X32" s="95"/>
-      <c r="Y32" s="96"/>
+      <c r="A32" s="98"/>
+      <c r="B32" s="100"/>
+      <c r="C32" s="100"/>
+      <c r="D32" s="100"/>
+      <c r="E32" s="100"/>
+      <c r="F32" s="100"/>
+      <c r="G32" s="100"/>
+      <c r="H32" s="100"/>
+      <c r="I32" s="100"/>
+      <c r="J32" s="100"/>
+      <c r="K32" s="100"/>
+      <c r="L32" s="100"/>
+      <c r="M32" s="100"/>
+      <c r="N32" s="100"/>
+      <c r="O32" s="100"/>
+      <c r="P32" s="100"/>
+      <c r="Q32" s="100"/>
+      <c r="R32" s="100"/>
+      <c r="S32" s="100"/>
+      <c r="T32" s="100"/>
+      <c r="U32" s="100"/>
+      <c r="V32" s="100"/>
+      <c r="W32" s="100"/>
+      <c r="X32" s="100"/>
+      <c r="Y32" s="106"/>
     </row>
     <row r="33" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A33" s="97"/>
+      <c r="A33" s="94"/>
       <c r="B33" s="62"/>
       <c r="C33" s="62"/>
       <c r="D33" s="62"/>
@@ -31692,37 +31140,37 @@
       <c r="V33" s="62"/>
       <c r="W33" s="62"/>
       <c r="X33" s="62"/>
-      <c r="Y33" s="98"/>
+      <c r="Y33" s="107"/>
     </row>
     <row r="34" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A34" s="93"/>
-      <c r="B34" s="95"/>
-      <c r="C34" s="95"/>
-      <c r="D34" s="95"/>
-      <c r="E34" s="95"/>
-      <c r="F34" s="95"/>
-      <c r="G34" s="95"/>
-      <c r="H34" s="95"/>
-      <c r="I34" s="95"/>
-      <c r="J34" s="95"/>
-      <c r="K34" s="95"/>
-      <c r="L34" s="95"/>
-      <c r="M34" s="95"/>
-      <c r="N34" s="95"/>
-      <c r="O34" s="95"/>
-      <c r="P34" s="95"/>
-      <c r="Q34" s="95"/>
-      <c r="R34" s="95"/>
-      <c r="S34" s="95"/>
-      <c r="T34" s="95"/>
-      <c r="U34" s="95"/>
-      <c r="V34" s="95"/>
-      <c r="W34" s="95"/>
-      <c r="X34" s="95"/>
-      <c r="Y34" s="96"/>
+      <c r="A34" s="98"/>
+      <c r="B34" s="100"/>
+      <c r="C34" s="100"/>
+      <c r="D34" s="100"/>
+      <c r="E34" s="100"/>
+      <c r="F34" s="100"/>
+      <c r="G34" s="100"/>
+      <c r="H34" s="100"/>
+      <c r="I34" s="100"/>
+      <c r="J34" s="100"/>
+      <c r="K34" s="100"/>
+      <c r="L34" s="100"/>
+      <c r="M34" s="100"/>
+      <c r="N34" s="100"/>
+      <c r="O34" s="100"/>
+      <c r="P34" s="100"/>
+      <c r="Q34" s="100"/>
+      <c r="R34" s="100"/>
+      <c r="S34" s="100"/>
+      <c r="T34" s="100"/>
+      <c r="U34" s="100"/>
+      <c r="V34" s="100"/>
+      <c r="W34" s="100"/>
+      <c r="X34" s="100"/>
+      <c r="Y34" s="106"/>
     </row>
     <row r="35" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A35" s="97"/>
+      <c r="A35" s="94"/>
       <c r="B35" s="62"/>
       <c r="C35" s="62"/>
       <c r="D35" s="62"/>
@@ -31746,72 +31194,72 @@
       <c r="V35" s="62"/>
       <c r="W35" s="62"/>
       <c r="X35" s="62"/>
-      <c r="Y35" s="98"/>
+      <c r="Y35" s="107"/>
     </row>
     <row r="36" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A36" s="93"/>
-      <c r="B36" s="95"/>
-      <c r="C36" s="95"/>
-      <c r="D36" s="95"/>
-      <c r="E36" s="95"/>
-      <c r="F36" s="95"/>
-      <c r="G36" s="95"/>
-      <c r="H36" s="95"/>
-      <c r="I36" s="95"/>
-      <c r="J36" s="95"/>
-      <c r="K36" s="95"/>
-      <c r="L36" s="95"/>
-      <c r="M36" s="95"/>
-      <c r="N36" s="95"/>
-      <c r="O36" s="95"/>
-      <c r="P36" s="95"/>
-      <c r="Q36" s="95"/>
-      <c r="R36" s="95"/>
-      <c r="S36" s="95"/>
-      <c r="T36" s="95"/>
-      <c r="U36" s="95"/>
-      <c r="V36" s="95"/>
-      <c r="W36" s="95"/>
-      <c r="X36" s="95"/>
-      <c r="Y36" s="96"/>
+      <c r="A36" s="98"/>
+      <c r="B36" s="100"/>
+      <c r="C36" s="100"/>
+      <c r="D36" s="100"/>
+      <c r="E36" s="100"/>
+      <c r="F36" s="100"/>
+      <c r="G36" s="100"/>
+      <c r="H36" s="100"/>
+      <c r="I36" s="100"/>
+      <c r="J36" s="100"/>
+      <c r="K36" s="100"/>
+      <c r="L36" s="100"/>
+      <c r="M36" s="100"/>
+      <c r="N36" s="100"/>
+      <c r="O36" s="100"/>
+      <c r="P36" s="100"/>
+      <c r="Q36" s="100"/>
+      <c r="R36" s="100"/>
+      <c r="S36" s="100"/>
+      <c r="T36" s="100"/>
+      <c r="U36" s="100"/>
+      <c r="V36" s="100"/>
+      <c r="W36" s="100"/>
+      <c r="X36" s="100"/>
+      <c r="Y36" s="106"/>
     </row>
     <row r="37" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A37" s="114"/>
-      <c r="B37" s="115"/>
-      <c r="C37" s="115"/>
-      <c r="D37" s="116">
+      <c r="A37" s="108"/>
+      <c r="B37" s="109"/>
+      <c r="C37" s="109"/>
+      <c r="D37" s="110">
         <f>+(D7+D8+D9+D10+D11+D12+D13+D14+D15+D16+D17+D18+D19+D20+D21+D22+D23+D24+D25+D26+D27+D28+D29+D30+D36)</f>
         <v>173760</v>
       </c>
-      <c r="E37" s="115"/>
-      <c r="F37" s="115"/>
-      <c r="G37" s="115"/>
-      <c r="H37" s="115"/>
-      <c r="I37" s="116">
+      <c r="E37" s="109"/>
+      <c r="F37" s="109"/>
+      <c r="G37" s="109"/>
+      <c r="H37" s="109"/>
+      <c r="I37" s="110">
         <f>+(I7+I8+I9+I10+I11+I12+I13+I14+I15+I16+I17+I18+I20+I19+I21+I22+I23+I24+I25+I26+I27+I29+I28+I30+I36)</f>
         <v>87240</v>
       </c>
-      <c r="J37" s="115"/>
-      <c r="K37" s="115"/>
-      <c r="L37" s="115"/>
-      <c r="M37" s="116">
-        <v>0</v>
-      </c>
-      <c r="N37" s="115"/>
-      <c r="O37" s="115"/>
-      <c r="P37" s="115"/>
-      <c r="Q37" s="117">
+      <c r="J37" s="109"/>
+      <c r="K37" s="109"/>
+      <c r="L37" s="109"/>
+      <c r="M37" s="110">
+        <v>0</v>
+      </c>
+      <c r="N37" s="109"/>
+      <c r="O37" s="109"/>
+      <c r="P37" s="109"/>
+      <c r="Q37" s="111">
         <f>SUM(Q7:Q36)</f>
         <v>0</v>
       </c>
-      <c r="R37" s="115"/>
-      <c r="S37" s="115"/>
-      <c r="T37" s="115"/>
-      <c r="U37" s="115"/>
-      <c r="V37" s="115"/>
-      <c r="W37" s="115"/>
-      <c r="X37" s="115"/>
-      <c r="Y37" s="118"/>
+      <c r="R37" s="109"/>
+      <c r="S37" s="109"/>
+      <c r="T37" s="109"/>
+      <c r="U37" s="109"/>
+      <c r="V37" s="109"/>
+      <c r="W37" s="109"/>
+      <c r="X37" s="109"/>
+      <c r="Y37" s="112"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Align shed layouts by hiding extra date columns and adjusting widths
Adjust scripts to hide specific columns and resize others in the spreadsheet to ensure visual consistency across all shed tabs.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: a3bb658e-c1b8-4d25-a4e2-55594f80be40
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: f0f7c297-ed2f-4f6d-9b96-de4a405b9f53
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9fb187d0-5a71-40d4-a291-96ab5e107c04/a3bb658e-c1b8-4d25-a4e2-55594f80be40/IeCay9D
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/silo-tracker/public/silo-mate-feed-program.xlsx
+++ b/artifacts/silo-tracker/public/silo-mate-feed-program.xlsx
@@ -21204,9 +21204,9 @@
   <sheetFormatPr defaultRowHeight="22.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25" defaultColWidth="14.6953125" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="5.52734375" style="62" customWidth="1"/>
-    <col min="2" max="2" width="16.5859375" style="62" customWidth="1"/>
+    <col min="2" max="2" width="55" style="62" customWidth="1"/>
     <col min="3" max="13" width="16.5859375" style="63" hidden="1" customWidth="1"/>
-    <col min="14" max="14" width="44.23046875" style="62" customWidth="1"/>
+    <col min="14" max="14" width="44.23046875" style="62" hidden="1" customWidth="1"/>
     <col min="15" max="15" width="14.5625" style="64" customWidth="1"/>
     <col min="16" max="16" width="17.6640625" style="64" customWidth="1"/>
     <col min="17" max="17" width="10.11328125" style="64" customWidth="1"/>

</xml_diff>

<commit_message>
Preserve original colours and update tab colours for feed program
Remove cell fill remapping logic from Excel styling script, preserving all original cell colours, fonts, and data. Update SHED tab colours to match reference file pattern and set specific tab colours for END and BATCH sheets.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: a3bb658e-c1b8-4d25-a4e2-55594f80be40
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: edcffb41-a2c5-45bd-a34e-68dcfcae4b57
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9fb187d0-5a71-40d4-a291-96ab5e107c04/a3bb658e-c1b8-4d25-a4e2-55594f80be40/IeCay9D
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/silo-tracker/public/silo-mate-feed-program.xlsx
+++ b/artifacts/silo-tracker/public/silo-mate-feed-program.xlsx
@@ -669,7 +669,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -678,12 +678,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF217346"/>
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
@@ -700,13 +702,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor theme="8" tint="0.7999816888943144"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.7999816888943144"/>
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -736,12 +738,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor indexed="9"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -749,12 +745,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="3" tint="0.8999908444471572"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1698,7 +1688,7 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1707,31 +1697,31 @@
     <xf numFmtId="1" fontId="7" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="7" fillId="7" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="7" fillId="6" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="9" fillId="7" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="9" fillId="6" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="9" fillId="7" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="9" fillId="6" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="7" fillId="7" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="7" fillId="6" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1746,28 +1736,28 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="6" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="12" fillId="6" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="7" fillId="7" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="7" fillId="6" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="7" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="7" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="7" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="7" fillId="6" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="7" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -2152,54 +2142,54 @@
     <xf numFmtId="0" fontId="25" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="12" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="26" fillId="12" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="26" fillId="12" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="26" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="26" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="27" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="12" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="12" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="28" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="25" fillId="9" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="9" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="13" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="12" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="13" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="12" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="13" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="13" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="30" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="13" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="13" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2210,12 +2200,39 @@
     <xf numFmtId="0" fontId="31" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="30" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="33" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="30" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
     <xf numFmtId="0" fontId="30" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2223,33 +2240,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="13" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="13" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2273,10 +2263,10 @@
     <xf numFmtId="0" fontId="30" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="30" fillId="13" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="30" fillId="13" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="30" fillId="16" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="30" fillId="14" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
@@ -2289,7 +2279,7 @@
     <xf numFmtId="0" fontId="36" fillId="8" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="37" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="38" fillId="8" borderId="51" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2327,7 +2317,7 @@
     <xf numFmtId="167" fontId="41" fillId="8" borderId="51" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="13" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="33" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="30" fillId="3" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2353,7 +2343,7 @@
     <xf numFmtId="167" fontId="30" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="13" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="33" fillId="8" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2369,7 +2359,7 @@
     <xf numFmtId="0" fontId="30" fillId="3" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="30" fillId="17" borderId="53" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="30" fillId="15" borderId="53" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2430,10 +2420,10 @@
     <xf numFmtId="2" fontId="30" fillId="8" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="13" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="167" fontId="30" fillId="8" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5453,7 +5443,7 @@
 <file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
-    <tabColor rgb="FF217346"/>
+    <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:AN78"/>
   <sheetFormatPr defaultRowHeight="22.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25" defaultColWidth="14.6953125" customHeight="1"/>
@@ -9416,7 +9406,7 @@
 <file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
-    <tabColor rgb="FF0070C0"/>
+    <tabColor rgb="FF00B0F0"/>
   </sheetPr>
   <dimension ref="A1:AN78"/>
   <sheetFormatPr defaultRowHeight="22.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25" defaultColWidth="14.6953125" customHeight="1"/>
@@ -21291,7 +21281,7 @@
 <file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
-    <tabColor rgb="FF217346"/>
+    <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:AY78"/>
   <sheetFormatPr defaultRowHeight="22.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25" defaultColWidth="14.6953125" customHeight="1"/>
@@ -26116,7 +26106,7 @@
 <file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
-    <tabColor rgb="FF0070C0"/>
+    <tabColor rgb="FF00B0F0"/>
   </sheetPr>
   <dimension ref="A1:AN78"/>
   <sheetFormatPr defaultRowHeight="22.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25" defaultColWidth="14.6953125" customHeight="1"/>
@@ -30077,7 +30067,7 @@
 <file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
-    <tabColor rgb="FF217346"/>
+    <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:AI39"/>
   <sheetFormatPr defaultRowHeight="12.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.15" customHeight="1"/>

</xml_diff>